<commit_message>
Replace banner photos with unclear rights and add image rights check
Swap two press photos (HG) and one unverified, likely AI-generated photo (PF)
for the businesses' own project photos. Add an Image Rights column and an
Image Rights Check tab listing source, evidence and verdict per photo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WnXcuRrGu4zGnnykNFmZUS
</commit_message>
<xml_diff>
--- a/deliverables/gbp-calendars/Harlingen-Glass-GBP-Monthly-Calendar-Nov-2026.xlsx
+++ b/deliverables/gbp-calendars/Harlingen-Glass-GBP-Monthly-Calendar-Nov-2026.xlsx
@@ -11,11 +11,12 @@
     <sheet name="harlingenglass.com" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Settings" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Banner &amp; Brand Kit" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="GBP Guidelines" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="QA Cross-Check" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Image Rights Check" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="GBP Guidelines" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="QA Cross-Check" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'harlingenglass.com'!$B$1:$P$23</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'harlingenglass.com'!$B$1:$Q$23</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="370">
   <si>
     <t xml:space="preserve">Week</t>
   </si>
@@ -66,6 +67,9 @@
   </si>
   <si>
     <t xml:space="preserve">Banner Photo Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Image Rights</t>
   </si>
   <si>
     <t xml:space="preserve">Offer Dates / Terms</t>
@@ -103,6 +107,9 @@
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/image00008.jpg</t>
   </si>
   <si>
+    <t xml:space="preserve">Business's own photo from its website (client to confirm ownership).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not Published</t>
   </si>
   <si>
@@ -447,7 +454,7 @@
     <t xml:space="preserve">2026-11-23_gbp-post-16_1200x900.png</t>
   </si>
   <si>
-    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/IDEA-Toros-College-Prep.jpg</t>
+    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/UTB-Kinesiology-Bldg.jpg</t>
   </si>
   <si>
     <t xml:space="preserve">Offer dates: Nov 23 to Dec 18, 2026 (confirm). Terms: assessment is free; installation quoted separately.</t>
@@ -496,6 +503,9 @@
     <t xml:space="preserve">https://unsplash.com/photos/_enXmoXudAk (Unsplash licence)</t>
   </si>
   <si>
+    <t xml:space="preserve">Unsplash License: free for commercial use, no permission or credit needed.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Happy Thanksgiving from Harlingen Glass &amp; Mirror</t>
   </si>
   <si>
@@ -903,15 +913,201 @@
     <t xml:space="preserve">Split photo, offer card, FAQ question, local spotlight, glass panel, 3-up compare, diagonal, frame, before/after, project spotlight, seasonal thank-you.</t>
   </si>
   <si>
+    <t xml:space="preserve">Image rights cross-check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every banner photo is either the business's own photo from its website or a free Unsplash photo. Checked Oct 26, 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Photo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source URL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Origin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence checked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verdict</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image00008.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Business website</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the harlingenglass.com media library (wp-content/uploads); No photographer credit, stock agency tag or watermark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OK: business's own photo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image00005.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20200117_133159154-scaled.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the harlingenglass.com media library (wp-content/uploads); Taken on a phone camera (motorola Moto E (4)): original photo, not stock; No photographer credit, stock agency tag or watermark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">McAllen-District-Office-12-04-08-001.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20231208_134141.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ShowerDoor-scaled.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/ShowerDoor-scaled.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image00004.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/image00004.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20231208_134144.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rio-Hondo-Middle-School-3.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image00003.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harlingen-Middle-School-Screw-Locations-Ext-Doors-011.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_0499-scaled.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the harlingenglass.com media library (wp-content/uploads); Taken on a phone camera (Apple iPhone 7): original photo, not stock; No photographer credit, stock agency tag or watermark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20231208_134139.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20231208_134148.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20231208_134134.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20200123_141554436-scaled.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UTB-Kinesiology-Bldg.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">McAllen-District-Office-12-04-08-002.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unsplash_cracked.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unsplash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Downloaded through the official Unsplash API; free photo, not Unsplash+; No photographer credit, stock agency tag or watermark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OK: royalty-free (Unsplash License)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">team_crop.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the harlingenglass.com media library (wp-content/uploads); Cropped from the team photo on the website; No photographer credit, stock agency tag or watermark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">before.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/before.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">after.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/after.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image00009.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45130555_1967058790260758_3379670728264646656_n.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/45130555_1967058790260758_3379670728264646656_n.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rio-Hondo-Middle-School-2.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/Rio-Hondo-Middle-School-2.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spi-Fire-Station-No-1.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/Spi-Fire-Station-No-1.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Photos OK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Photos removed during the check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Photo removed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaced with</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDEA-Toros-College-Prep-Front.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Credited to a press photographer (Jose Aldape) and carries a Texas Border Business watermark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rio-Hondo-Middle-School-3.jpg (own project photo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDEA-Toros-College-Prep.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same press photo series of a third-party school brand; ownership unclear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UTB-Kinesiology-Bldg.jpg (own project photo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: photos on the business's own website are treated as owned by the business. Ask the client to confirm they took these photos or hold the rights. Unsplash photos can be used commercially without credit, but do not show people or brands in a way that suggests endorsement.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Google Business Profile post rules applied to this calendar</t>
   </si>
   <si>
     <t xml:space="preserve">Every post and banner was written and checked against these rules.</t>
   </si>
   <si>
-    <t xml:space="preserve">#</t>
-  </si>
-  <si>
     <t xml:space="preserve">How this calendar follows it</t>
   </si>
   <si>
@@ -1015,9 +1211,6 @@
   </si>
   <si>
     <t xml:space="preserve">Formulas re-check every post when copy or links change. Every row should read Pass before scheduling.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date</t>
   </si>
   <si>
     <t xml:space="preserve">Characters</t>
@@ -2414,7 +2607,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:P23"/>
+  <dimension ref="B1:Q23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2431,8 +2624,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2481,6 +2674,9 @@
       <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="Q1" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="n">
@@ -2494,19 +2690,19 @@
         <v>Mon</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J2" s="5" t="str">
         <f aca="false">I2&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C13</f>
@@ -2514,17 +2710,20 @@
       </c>
       <c r="K2" s="4"/>
       <c r="L2" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="O2" s="4"/>
-      <c r="P2" s="2" t="s">
         <v>23</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2539,19 +2738,19 @@
         <v>Tue</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J3" s="5" t="str">
         <f aca="false">I3&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C14</f>
@@ -2559,19 +2758,22 @@
       </c>
       <c r="K3" s="4"/>
       <c r="L3" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2586,19 +2788,19 @@
         <v>Wed</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J4" s="5" t="str">
         <f aca="false">I4&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C15</f>
@@ -2606,17 +2808,20 @@
       </c>
       <c r="K4" s="4"/>
       <c r="L4" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="O4" s="4"/>
-      <c r="P4" s="2" t="s">
-        <v>23</v>
+        <v>40</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2631,19 +2836,19 @@
         <v>Thu</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J5" s="5" t="str">
         <f aca="false">I5&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C16</f>
@@ -2651,17 +2856,20 @@
       </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="O5" s="4"/>
-      <c r="P5" s="2" t="s">
-        <v>23</v>
+        <v>47</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2676,19 +2884,19 @@
         <v>Fri</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J6" s="5" t="str">
         <f aca="false">I6&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C17</f>
@@ -2696,17 +2904,20 @@
       </c>
       <c r="K6" s="4"/>
       <c r="L6" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="O6" s="4"/>
-      <c r="P6" s="2" t="s">
-        <v>23</v>
+        <v>54</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2721,19 +2932,19 @@
         <v>Mon</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J7" s="5" t="str">
         <f aca="false">I7&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C18</f>
@@ -2741,17 +2952,20 @@
       </c>
       <c r="K7" s="4"/>
       <c r="L7" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="O7" s="4"/>
-      <c r="P7" s="2" t="s">
-        <v>23</v>
+        <v>59</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2766,19 +2980,19 @@
         <v>Tue</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J8" s="5" t="str">
         <f aca="false">I8&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C19</f>
@@ -2786,17 +3000,20 @@
       </c>
       <c r="K8" s="4"/>
       <c r="L8" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="O8" s="4"/>
-      <c r="P8" s="2" t="s">
-        <v>23</v>
+        <v>65</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2811,19 +3028,19 @@
         <v>Wed</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J9" s="5" t="str">
         <f aca="false">I9&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C20</f>
@@ -2831,17 +3048,20 @@
       </c>
       <c r="K9" s="4"/>
       <c r="L9" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="O9" s="4"/>
-      <c r="P9" s="2" t="s">
-        <v>23</v>
+        <v>70</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2856,19 +3076,19 @@
         <v>Thu</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J10" s="5" t="str">
         <f aca="false">I10&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C21</f>
@@ -2876,17 +3096,20 @@
       </c>
       <c r="K10" s="4"/>
       <c r="L10" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="O10" s="4"/>
-      <c r="P10" s="2" t="s">
-        <v>23</v>
+        <v>75</v>
+      </c>
+      <c r="O10" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2901,19 +3124,19 @@
         <v>Fri</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="J11" s="5" t="str">
         <f aca="false">I11&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C22</f>
@@ -2921,17 +3144,20 @@
       </c>
       <c r="K11" s="4"/>
       <c r="L11" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="O11" s="4"/>
-      <c r="P11" s="2" t="s">
-        <v>23</v>
+        <v>81</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P11" s="4"/>
+      <c r="Q11" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2946,19 +3172,19 @@
         <v>Mon</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J12" s="5" t="str">
         <f aca="false">I12&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C23</f>
@@ -2966,17 +3192,20 @@
       </c>
       <c r="K12" s="4"/>
       <c r="L12" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="O12" s="4"/>
-      <c r="P12" s="2" t="s">
-        <v>23</v>
+        <v>87</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2991,19 +3220,19 @@
         <v>Tue</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="J13" s="5" t="str">
         <f aca="false">I13&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C24</f>
@@ -3011,17 +3240,20 @@
       </c>
       <c r="K13" s="4"/>
       <c r="L13" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="M13" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="N13" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="O13" s="4"/>
-      <c r="P13" s="2" t="s">
-        <v>23</v>
+        <v>93</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3036,19 +3268,19 @@
         <v>Wed</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J14" s="5" t="str">
         <f aca="false">I14&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C25</f>
@@ -3056,17 +3288,20 @@
       </c>
       <c r="K14" s="4"/>
       <c r="L14" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="M14" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="O14" s="4"/>
-      <c r="P14" s="2" t="s">
-        <v>23</v>
+        <v>98</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P14" s="4"/>
+      <c r="Q14" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3081,19 +3316,19 @@
         <v>Thu</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J15" s="5" t="str">
         <f aca="false">I15&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C26</f>
@@ -3101,17 +3336,20 @@
       </c>
       <c r="K15" s="4"/>
       <c r="L15" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="M15" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="N15" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="O15" s="4"/>
-      <c r="P15" s="2" t="s">
-        <v>23</v>
+        <v>103</v>
+      </c>
+      <c r="O15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3126,19 +3364,19 @@
         <v>Fri</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J16" s="5" t="str">
         <f aca="false">I16&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C27</f>
@@ -3146,17 +3384,20 @@
       </c>
       <c r="K16" s="4"/>
       <c r="L16" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="M16" s="4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="N16" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="O16" s="4"/>
-      <c r="P16" s="2" t="s">
-        <v>23</v>
+        <v>108</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P16" s="4"/>
+      <c r="Q16" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3171,19 +3412,19 @@
         <v>Mon</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J17" s="5" t="str">
         <f aca="false">I17&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C28</f>
@@ -3191,19 +3432,22 @@
       </c>
       <c r="K17" s="4"/>
       <c r="L17" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="M17" s="4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="N17" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="O17" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="P17" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="P17" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q17" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3218,19 +3462,19 @@
         <v>Tue</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="J18" s="5" t="str">
         <f aca="false">I18&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C29</f>
@@ -3238,17 +3482,20 @@
       </c>
       <c r="K18" s="4"/>
       <c r="L18" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="M18" s="4" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N18" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="O18" s="4"/>
-      <c r="P18" s="2" t="s">
-        <v>23</v>
+        <v>119</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P18" s="4"/>
+      <c r="Q18" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3263,19 +3510,19 @@
         <v>Wed</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="J19" s="5" t="str">
         <f aca="false">I19&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C30</f>
@@ -3283,17 +3530,20 @@
       </c>
       <c r="K19" s="4"/>
       <c r="L19" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="M19" s="4" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="N19" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="O19" s="4"/>
-      <c r="P19" s="2" t="s">
-        <v>23</v>
+        <v>125</v>
+      </c>
+      <c r="O19" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="P19" s="4"/>
+      <c r="Q19" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3308,19 +3558,19 @@
         <v>Thu</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J20" s="5" t="str">
         <f aca="false">I20&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C31</f>
@@ -3328,17 +3578,20 @@
       </c>
       <c r="K20" s="4"/>
       <c r="L20" s="4" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="M20" s="4" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="N20" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="O20" s="4"/>
-      <c r="P20" s="2" t="s">
-        <v>23</v>
+        <v>131</v>
+      </c>
+      <c r="O20" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P20" s="4"/>
+      <c r="Q20" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3353,19 +3606,19 @@
         <v>Fri</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J21" s="5" t="str">
         <f aca="false">I21&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C32</f>
@@ -3373,19 +3626,22 @@
       </c>
       <c r="K21" s="4"/>
       <c r="L21" s="4" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="M21" s="4" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N21" s="4" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O21" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="P21" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="P21" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q21" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3400,19 +3656,19 @@
         <v>Mon</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="J22" s="5" t="str">
         <f aca="false">I22&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C33</f>
@@ -3420,17 +3676,20 @@
       </c>
       <c r="K22" s="4"/>
       <c r="L22" s="4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="M22" s="4" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="N22" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="O22" s="4"/>
-      <c r="P22" s="2" t="s">
-        <v>23</v>
+        <v>142</v>
+      </c>
+      <c r="O22" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P22" s="4"/>
+      <c r="Q22" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3445,19 +3704,19 @@
         <v>Tue</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="J23" s="5" t="str">
         <f aca="false">I23&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C34</f>
@@ -3465,23 +3724,26 @@
       </c>
       <c r="K23" s="4"/>
       <c r="L23" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="M23" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="N23" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="O23" s="4"/>
-      <c r="P23" s="2" t="s">
-        <v>23</v>
+        <v>147</v>
+      </c>
+      <c r="O23" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P23" s="4"/>
+      <c r="Q23" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:P23"/>
+  <autoFilter ref="B1:Q23"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P2:P23" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="Q2:Q23" type="list">
       <formula1>"Not Published,Scheduled,Published"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3511,80 +3773,80 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="8" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="9" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="8" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>4</v>
@@ -3595,7 +3857,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D13" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F2</f>
@@ -3607,7 +3869,7 @@
         <v>2</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D14" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F3</f>
@@ -3619,7 +3881,7 @@
         <v>3</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D15" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F4</f>
@@ -3631,7 +3893,7 @@
         <v>4</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D16" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F5</f>
@@ -3643,7 +3905,7 @@
         <v>5</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D17" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F6</f>
@@ -3655,7 +3917,7 @@
         <v>6</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D18" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F7</f>
@@ -3667,7 +3929,7 @@
         <v>7</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D19" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F8</f>
@@ -3679,7 +3941,7 @@
         <v>8</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D20" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F9</f>
@@ -3691,7 +3953,7 @@
         <v>9</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D21" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F10</f>
@@ -3703,7 +3965,7 @@
         <v>10</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D22" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F11</f>
@@ -3715,7 +3977,7 @@
         <v>11</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D23" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F12</f>
@@ -3727,7 +3989,7 @@
         <v>12</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D24" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F13</f>
@@ -3739,7 +4001,7 @@
         <v>13</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D25" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F14</f>
@@ -3751,7 +4013,7 @@
         <v>14</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D26" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F15</f>
@@ -3763,7 +4025,7 @@
         <v>15</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D27" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F16</f>
@@ -3775,7 +4037,7 @@
         <v>16</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D28" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F17</f>
@@ -3787,7 +4049,7 @@
         <v>17</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D29" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F18</f>
@@ -3799,7 +4061,7 @@
         <v>18</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D30" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F19</f>
@@ -3811,7 +4073,7 @@
         <v>19</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D31" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F20</f>
@@ -3823,7 +4085,7 @@
         <v>20</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D32" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F21</f>
@@ -3835,7 +4097,7 @@
         <v>21</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D33" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F22</f>
@@ -3847,7 +4109,7 @@
         <v>22</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D34" s="4" t="str">
         <f aca="false">'harlingenglass.com'!F23</f>
@@ -3883,262 +4145,262 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="8" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="4" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="4" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="4" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="9" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="4" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="4" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="4" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="F17" s="13"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="4" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="C18" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>228</v>
-      </c>
       <c r="E18" s="4" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="F18" s="14"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F19" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="9" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="8" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="4" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="4" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="4" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="4" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -4157,219 +4419,731 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>254</v>
+        <v>166</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>238</v>
+        <v>257</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>256</v>
+        <v>259</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>257</v>
+      <c r="B5" s="3" t="n">
+        <v>46328</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>23</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>260</v>
+      <c r="B6" s="3" t="n">
+        <v>46329</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>259</v>
+        <v>33</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>262</v>
+      <c r="B7" s="3" t="n">
+        <v>46330</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F7" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="n">
+        <v>46331</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>265</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="G8" s="4" t="s">
         <v>266</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>268</v>
+      <c r="B9" s="3" t="n">
+        <v>46332</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>54</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>270</v>
+      <c r="B10" s="3" t="n">
+        <v>46335</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>273</v>
+        <v>6</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>46335</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>274</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>275</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>275</v>
+        <v>6</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>46335</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>276</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>277</v>
+        <v>98</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>278</v>
+        <v>7</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>46336</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>277</v>
+        <v>65</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>280</v>
+        <v>8</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>46337</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>277</v>
+        <v>70</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>282</v>
+        <v>9</v>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>46338</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>75</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>284</v>
+        <v>10</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>46339</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>259</v>
+        <v>81</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>46342</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>46343</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B19" s="3" t="n">
+        <v>46344</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>46345</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>46346</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>46349</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="D22" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>46350</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>287</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>267</v>
+      <c r="D23" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>46351</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>46352</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>46353</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>46353</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>46356</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>46357</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>46357</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>46357</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="B33" s="9" t="str">
+        <f aca="false">COUNTIF(G5:G31,"OK*")&amp;" of "&amp;COUNTA(G5:G31)</f>
+        <v>27 of 27</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="8" t="s">
+        <v>307</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="s">
+        <v>317</v>
       </c>
     </row>
   </sheetData>
@@ -4384,6 +5158,237 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>307</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>320</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>332</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
@@ -4405,53 +5410,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>288</v>
+        <v>353</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>289</v>
+        <v>354</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>290</v>
+        <v>257</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>291</v>
+        <v>355</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>292</v>
+        <v>356</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>293</v>
+        <v>357</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>294</v>
+        <v>358</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>295</v>
+        <v>359</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>296</v>
+        <v>360</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>297</v>
+        <v>361</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>298</v>
+        <v>362</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>299</v>
+        <v>363</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>300</v>
+        <v>364</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>301</v>
+        <v>365</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5622,7 +6627,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>302</v>
+        <v>366</v>
       </c>
       <c r="B28" s="9" t="str">
         <f aca="false">COUNTIF(M5:M26,"Pass")&amp;" of "&amp;COUNTA(A5:A26)</f>
@@ -5631,7 +6636,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>303</v>
+        <v>367</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5639,12 +6644,12 @@
         <v>3</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>304</v>
+        <v>368</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B32" s="2" t="n">
         <f aca="false">COUNTIF('harlingenglass.com'!$E$2:$E$23,"Service")</f>
@@ -5653,7 +6658,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B33" s="2" t="n">
         <f aca="false">COUNTIF('harlingenglass.com'!$E$2:$E$23,"FAQ")</f>
@@ -5662,7 +6667,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B34" s="2" t="n">
         <f aca="false">COUNTIF('harlingenglass.com'!$E$2:$E$23,"Local")</f>
@@ -5671,7 +6676,7 @@
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B35" s="2" t="n">
         <f aca="false">COUNTIF('harlingenglass.com'!$E$2:$E$23,"Promotional")</f>
@@ -5680,7 +6685,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>305</v>
+        <v>369</v>
       </c>
       <c r="B36" s="2" t="n">
         <f aca="false">SUM(B32:B35)</f>

</xml_diff>

<commit_message>
Fix banner alignment and match every photo to its headline
Vertically centre text blocks, stop offer highlights overlapping lines,
keep hyphenated words together and auto-shrink long headlines, clear the
logo/tag overlap on the comparison layout, and re-crop photos. Swap
photos that did not match the post topic (foggy window, storm-damaged
fence, repair vs replace, SimTek stone look) for relevant site or
Unsplash photos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WnXcuRrGu4zGnnykNFmZUS
</commit_message>
<xml_diff>
--- a/deliverables/gbp-calendars/Harlingen-Glass-GBP-Monthly-Calendar-Nov-2026.xlsx
+++ b/deliverables/gbp-calendars/Harlingen-Glass-GBP-Monthly-Calendar-Nov-2026.xlsx
@@ -166,7 +166,10 @@
     <t xml:space="preserve">2026-11-04_gbp-post-03_1200x900.png</t>
   </si>
   <si>
-    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/IMG_20200117_133159154-scaled.jpg</t>
+    <t xml:space="preserve">https://unsplash.com/photos/9EyiD1RRYRs (Unsplash licence)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unsplash License: free for commercial use, no permission or credit needed.</t>
   </si>
   <si>
     <t xml:space="preserve">Local</t>
@@ -320,7 +323,7 @@
   </si>
   <si>
     <t xml:space="preserve">Tag: Commercial Glazing
-Headline: Your Storefront Is Your First Impression
+Headline: First Impressions Start at Your Storefront
 Sub-line: Storefronts, entry doors and multi-story glazing
 Button: Request an Assessment</t>
   </si>
@@ -503,9 +506,6 @@
     <t xml:space="preserve">https://unsplash.com/photos/_enXmoXudAk (Unsplash licence)</t>
   </si>
   <si>
-    <t xml:space="preserve">Unsplash License: free for commercial use, no permission or credit needed.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Happy Thanksgiving from Harlingen Glass &amp; Mirror</t>
   </si>
   <si>
@@ -952,60 +952,69 @@
     <t xml:space="preserve">image00005.jpg</t>
   </si>
   <si>
-    <t xml:space="preserve">IMG_20200117_133159154-scaled.jpg</t>
+    <t xml:space="preserve">unsplash_9EyiD1RRYRs.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unsplash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Downloaded through the official Unsplash API; free photo, not Unsplash+; No photographer credit, stock agency tag or watermark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OK: royalty-free (Unsplash License)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">McAllen-District-Office-12-04-08-001.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20231208_134141.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ShowerDoor-scaled.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/ShowerDoor-scaled.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image00004.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/image00004.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20231208_134144.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rio-Hondo-Middle-School-3.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image00003.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harlingen-Middle-School-Screw-Locations-Ext-Doors-011.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_0499-scaled.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the harlingenglass.com media library (wp-content/uploads); Taken on a phone camera (Apple iPhone 7): original photo, not stock; No photographer credit, stock agency tag or watermark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20231208_134139.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20231208_134148.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20231208_134134.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMG_20200123_141554436-scaled.jpg</t>
   </si>
   <si>
     <t xml:space="preserve">In the harlingenglass.com media library (wp-content/uploads); Taken on a phone camera (motorola Moto E (4)): original photo, not stock; No photographer credit, stock agency tag or watermark</t>
   </si>
   <si>
-    <t xml:space="preserve">McAllen-District-Office-12-04-08-001.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMG_20231208_134141.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ShowerDoor-scaled.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/ShowerDoor-scaled.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">image00004.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/image00004.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMG_20231208_134144.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rio-Hondo-Middle-School-3.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">image00003.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harlingen-Middle-School-Screw-Locations-Ext-Doors-011.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMG_0499-scaled.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In the harlingenglass.com media library (wp-content/uploads); Taken on a phone camera (Apple iPhone 7): original photo, not stock; No photographer credit, stock agency tag or watermark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMG_20231208_134139.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMG_20231208_134148.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMG_20231208_134134.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMG_20200123_141554436-scaled.jpg</t>
-  </si>
-  <si>
     <t xml:space="preserve">UTB-Kinesiology-Bldg.jpg</t>
   </si>
   <si>
@@ -1013,15 +1022,6 @@
   </si>
   <si>
     <t xml:space="preserve">unsplash_cracked.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unsplash</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Downloaded through the official Unsplash API; free photo, not Unsplash+; No photographer credit, stock agency tag or watermark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OK: royalty-free (Unsplash License)</t>
   </si>
   <si>
     <t xml:space="preserve">team_crop.jpg</t>
@@ -2817,7 +2817,7 @@
         <v>40</v>
       </c>
       <c r="O4" s="4" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="P4" s="4"/>
       <c r="Q4" s="2" t="s">
@@ -2836,19 +2836,19 @@
         <v>Thu</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J5" s="5" t="str">
         <f aca="false">I5&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C16</f>
@@ -2856,13 +2856,13 @@
       </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O5" s="4" t="s">
         <v>24</v>
@@ -2887,16 +2887,16 @@
         <v>16</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J6" s="5" t="str">
         <f aca="false">I6&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C17</f>
@@ -2904,13 +2904,13 @@
       </c>
       <c r="K6" s="4"/>
       <c r="L6" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O6" s="4" t="s">
         <v>24</v>
@@ -2935,16 +2935,16 @@
         <v>35</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J7" s="5" t="str">
         <f aca="false">I7&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C18</f>
@@ -2952,13 +2952,13 @@
       </c>
       <c r="K7" s="4"/>
       <c r="L7" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="O7" s="4" t="s">
         <v>24</v>
@@ -2983,16 +2983,16 @@
         <v>16</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J8" s="5" t="str">
         <f aca="false">I8&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C19</f>
@@ -3000,13 +3000,13 @@
       </c>
       <c r="K8" s="4"/>
       <c r="L8" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O8" s="4" t="s">
         <v>24</v>
@@ -3028,13 +3028,13 @@
         <v>Wed</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>19</v>
@@ -3048,13 +3048,13 @@
       </c>
       <c r="K9" s="4"/>
       <c r="L9" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O9" s="4" t="s">
         <v>24</v>
@@ -3079,16 +3079,16 @@
         <v>35</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J10" s="5" t="str">
         <f aca="false">I10&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C21</f>
@@ -3096,13 +3096,13 @@
       </c>
       <c r="K10" s="4"/>
       <c r="L10" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O10" s="4" t="s">
         <v>24</v>
@@ -3127,16 +3127,16 @@
         <v>16</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J11" s="5" t="str">
         <f aca="false">I11&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C22</f>
@@ -3144,13 +3144,13 @@
       </c>
       <c r="K11" s="4"/>
       <c r="L11" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O11" s="4" t="s">
         <v>24</v>
@@ -3175,16 +3175,16 @@
         <v>26</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J12" s="5" t="str">
         <f aca="false">I12&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C23</f>
@@ -3192,13 +3192,13 @@
       </c>
       <c r="K12" s="4"/>
       <c r="L12" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O12" s="4" t="s">
         <v>24</v>
@@ -3223,16 +3223,16 @@
         <v>16</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J13" s="5" t="str">
         <f aca="false">I13&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C24</f>
@@ -3240,13 +3240,13 @@
       </c>
       <c r="K13" s="4"/>
       <c r="L13" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="M13" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="N13" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="O13" s="4" t="s">
         <v>24</v>
@@ -3271,16 +3271,16 @@
         <v>35</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J14" s="5" t="str">
         <f aca="false">I14&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C25</f>
@@ -3288,13 +3288,13 @@
       </c>
       <c r="K14" s="4"/>
       <c r="L14" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="M14" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="O14" s="4" t="s">
         <v>24</v>
@@ -3316,13 +3316,13 @@
         <v>Thu</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>19</v>
@@ -3336,13 +3336,13 @@
       </c>
       <c r="K15" s="4"/>
       <c r="L15" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M15" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="N15" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O15" s="4" t="s">
         <v>24</v>
@@ -3367,10 +3367,10 @@
         <v>16</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>19</v>
@@ -3384,13 +3384,13 @@
       </c>
       <c r="K16" s="4"/>
       <c r="L16" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M16" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N16" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="O16" s="4" t="s">
         <v>24</v>
@@ -3415,16 +3415,16 @@
         <v>26</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J17" s="5" t="str">
         <f aca="false">I17&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C28</f>
@@ -3432,19 +3432,19 @@
       </c>
       <c r="K17" s="4"/>
       <c r="L17" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M17" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="N17" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="O17" s="4" t="s">
         <v>24</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q17" s="2" t="s">
         <v>25</v>
@@ -3465,16 +3465,16 @@
         <v>16</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J18" s="5" t="str">
         <f aca="false">I18&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C29</f>
@@ -3482,13 +3482,13 @@
       </c>
       <c r="K18" s="4"/>
       <c r="L18" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="M18" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="N18" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="O18" s="4" t="s">
         <v>24</v>
@@ -3513,16 +3513,16 @@
         <v>35</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J19" s="5" t="str">
         <f aca="false">I19&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C30</f>
@@ -3530,16 +3530,16 @@
       </c>
       <c r="K19" s="4"/>
       <c r="L19" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="M19" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N19" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>126</v>
+        <v>41</v>
       </c>
       <c r="P19" s="4"/>
       <c r="Q19" s="2" t="s">
@@ -3558,7 +3558,7 @@
         <v>Thu</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>127</v>
@@ -3570,7 +3570,7 @@
         <v>19</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J20" s="5" t="str">
         <f aca="false">I20&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C31</f>
@@ -3618,7 +3618,7 @@
         <v>29</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J21" s="5" t="str">
         <f aca="false">I21&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C32</f>
@@ -3668,7 +3668,7 @@
         <v>19</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J22" s="5" t="str">
         <f aca="false">I22&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C33</f>
@@ -3704,7 +3704,7 @@
         <v>Tue</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>143</v>
@@ -3716,7 +3716,7 @@
         <v>19</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J23" s="5" t="str">
         <f aca="false">I23&amp;"?utm_source="&amp;Settings!$C$5&amp;"&amp;utm_medium="&amp;Settings!$C$6&amp;"&amp;utm_campaign="&amp;Settings!$C$7&amp;"&amp;utm_content="&amp;Settings!C34</f>
@@ -4510,7 +4510,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="n">
         <v>3</v>
       </c>
@@ -4524,13 +4524,13 @@
         <v>40</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4541,10 +4541,10 @@
         <v>46331</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>264</v>
@@ -4564,10 +4564,10 @@
         <v>46332</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>264</v>
@@ -4587,10 +4587,10 @@
         <v>46335</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>264</v>
@@ -4610,10 +4610,10 @@
         <v>46335</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>264</v>
@@ -4633,10 +4633,10 @@
         <v>46335</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>264</v>
@@ -4656,10 +4656,10 @@
         <v>46336</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>264</v>
@@ -4679,10 +4679,10 @@
         <v>46337</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>264</v>
@@ -4702,10 +4702,10 @@
         <v>46338</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>264</v>
@@ -4725,16 +4725,16 @@
         <v>46339</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>264</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="G16" s="4" t="s">
         <v>266</v>
@@ -4748,10 +4748,10 @@
         <v>46342</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>264</v>
@@ -4771,10 +4771,10 @@
         <v>46343</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>264</v>
@@ -4794,10 +4794,10 @@
         <v>46344</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>264</v>
@@ -4817,10 +4817,10 @@
         <v>46345</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>264</v>
@@ -4840,16 +4840,16 @@
         <v>46346</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>264</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>266</v>
@@ -4863,10 +4863,10 @@
         <v>46349</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>264</v>
@@ -4886,10 +4886,10 @@
         <v>46350</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>264</v>
@@ -4909,19 +4909,19 @@
         <v>46351</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>289</v>
+        <v>269</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>291</v>
+        <v>271</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6667,7 +6667,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B34" s="2" t="n">
         <f aca="false">COUNTIF('harlingenglass.com'!$E$2:$E$23,"Local")</f>

</xml_diff>

<commit_message>
Cross-check calendar offers against both websites
Add a Website Offers Check tab listing every live offer with its exact
wording, page and the posts that use it. Reword the Preferred Fence
design post (the site offers free estimates, not a free consultation),
add the stated financing and Ameristar 20-year warranty to the posts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WnXcuRrGu4zGnnykNFmZUS
</commit_message>
<xml_diff>
--- a/deliverables/gbp-calendars/Harlingen-Glass-GBP-Monthly-Calendar-Nov-2026.xlsx
+++ b/deliverables/gbp-calendars/Harlingen-Glass-GBP-Monthly-Calendar-Nov-2026.xlsx
@@ -12,8 +12,9 @@
     <sheet name="Settings" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Banner &amp; Brand Kit" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Image Rights Check" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="GBP Guidelines" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="QA Cross-Check" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Website Offers Check" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="GBP Guidelines" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="QA Cross-Check" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'harlingenglass.com'!$B$1:$Q$23</definedName>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="411">
   <si>
     <t xml:space="preserve">Week</t>
   </si>
@@ -1100,6 +1101,129 @@
   </si>
   <si>
     <t xml:space="preserve">Note: photos on the business's own website are treated as owned by the business. Ask the client to confirm they took these photos or hold the rights. Unsplash photos can be used commercially without credit, but do not show people or brands in a way that suggests endorsement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offers on the website vs. this calendar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every page of harlingenglass.com was checked on Oct 26, 2026. Posts only promote offers the website states.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exact wording on the website</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used in post #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 3 windows, get the 4th free</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy 3 Windows, Get the 4th Window FREE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 (Offer post)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live on the website. No dates or terms are shown, so confirm the end date, eligible window types and whether it combines with financing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free window inspection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get Your Free Window Inspection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2, 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used as the button text and in the post copy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free bathroom glass consultation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get A Free Consultation! No cost, no pressure, just expert advice and a clear quote!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5, 20 (Offer post)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live on the website. The page also says 'Appointments Filling Fast'; the calendar does not repeat that urgency claim.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financing through Synchrony Bank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harlingen Glass is proud to announce that we have partnered with Synchrony bank to bring financing options</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://harlingenglass.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5, 11, 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bathroom page also shows 'Financing Available'. Rates and terms are not on the website, so posts do not quote any.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free 3M security film assessment (schools)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get Your Free Security Film Assessment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9, 16 (Offer post)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live on the website. Installation is quoted separately.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free estimate / free quote</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET A FREE ESTIMATE! / Get A Free Quote Today</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://harlingenglass.com/ and /service/interior/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1, 12, 21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General offer; used as button text.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warranty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manufacturer warranty of up to 3 years as well as an installation warranty of 1 year for specific products</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Post repeats the 'specific products' limit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emergency and after-hours service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We also offer emergency and after-hours services</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://harlingenglass.com/blog/preparing-your-home-for-summer-with-smart-glass-upgrades/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only stated in a blog post. Confirm with the client before promoting it.</t>
   </si>
   <si>
     <t xml:space="preserve">Google Business Profile post rules applied to this calendar</t>
@@ -5162,13 +5286,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5186,13 +5312,19 @@
         <v>307</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>241</v>
+        <v>320</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>321</v>
+        <v>322</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5200,55 +5332,79 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>30</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>30</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>52</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>332</v>
+        <v>338</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5256,13 +5412,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>332</v>
+        <v>63</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5270,13 +5432,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>337</v>
+        <v>347</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5284,97 +5452,39 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>338</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>339</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E11" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>340</v>
+        <v>354</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>341</v>
+        <v>355</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>343</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>344</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>345</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>346</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>347</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>348</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>349</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>350</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>351</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>352</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>332</v>
+        <v>356</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -5389,6 +5499,237 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>307</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>373</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
@@ -5410,12 +5751,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>353</v>
+        <v>394</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>354</v>
+        <v>395</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5426,37 +5767,37 @@
         <v>257</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>355</v>
+        <v>396</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>356</v>
+        <v>397</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>357</v>
+        <v>398</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>358</v>
+        <v>399</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>359</v>
+        <v>400</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>360</v>
+        <v>401</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>361</v>
+        <v>402</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>362</v>
+        <v>403</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>363</v>
+        <v>404</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>364</v>
+        <v>405</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>365</v>
+        <v>406</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6627,7 +6968,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>366</v>
+        <v>407</v>
       </c>
       <c r="B28" s="9" t="str">
         <f aca="false">COUNTIF(M5:M26,"Pass")&amp;" of "&amp;COUNTA(A5:A26)</f>
@@ -6636,7 +6977,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>367</v>
+        <v>408</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6644,7 +6985,7 @@
         <v>3</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>368</v>
+        <v>409</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6685,7 +7026,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>369</v>
+        <v>410</v>
       </c>
       <c r="B36" s="2" t="n">
         <f aca="false">SUM(B32:B35)</f>

</xml_diff>

<commit_message>
Use an AI-generated stone-look fence image for the SimTek banner
No SimTek install photo exists on the website, so the banner uses an
Ideogram illustration, labelled as AI-generated in the Image Rights
column and check tab.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WnXcuRrGu4zGnnykNFmZUS
</commit_message>
<xml_diff>
--- a/deliverables/gbp-calendars/Harlingen-Glass-GBP-Monthly-Calendar-Nov-2026.xlsx
+++ b/deliverables/gbp-calendars/Harlingen-Glass-GBP-Monthly-Calendar-Nov-2026.xlsx
@@ -1100,7 +1100,7 @@
     <t xml:space="preserve">UTB-Kinesiology-Bldg.jpg (own project photo)</t>
   </si>
   <si>
-    <t xml:space="preserve">Note: photos on the business's own website are treated as owned by the business. Ask the client to confirm they took these photos or hold the rights. Unsplash photos can be used commercially without credit, but do not show people or brands in a way that suggests endorsement.</t>
+    <t xml:space="preserve">Note: photos on the business's own website are treated as owned by the business. Ask the client to confirm they took these photos or hold the rights. Unsplash photos can be used commercially without credit, but do not show people or brands in a way that suggests endorsement. AI-generated images are illustrations only: never present them as the client's own finished work, and get client approval before posting.</t>
   </si>
   <si>
     <t xml:space="preserve">Offers on the website vs. this calendar</t>
@@ -1322,7 +1322,7 @@
     <t xml:space="preserve">Photos must follow the photo policy: real, relevant to the business, not misleading.</t>
   </si>
   <si>
-    <t xml:space="preserve">Every banner uses a real photo from the business's own website (one HG post uses a licensed Unsplash photo). Overlay text is short (headline plus one line), with no phone numbers, emails, prices or claims that are not on the website.</t>
+    <t xml:space="preserve">Banners use the business's own website photos where one fits the topic. Where none fits, a free Unsplash photo is used, and one Preferred Fence banner (SimTek) uses an AI-generated illustration, marked on the Image Rights Check tab. Overlay text is short (headline plus one line), with no phone numbers, emails, prices or claims that are not on the website.</t>
   </si>
   <si>
     <t xml:space="preserve">Recommended post image: JPG or PNG, 10 KB to 5 MB, at least 400 x 300 px, 4:3 ratio displays best.</t>
@@ -5690,7 +5690,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="n">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
Link each banner to its Google Drive copy in the calendar sheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WnXcuRrGu4zGnnykNFmZUS
</commit_message>
<xml_diff>
--- a/deliverables/gbp-calendars/Harlingen-Glass-GBP-Monthly-Calendar-Nov-2026.xlsx
+++ b/deliverables/gbp-calendars/Harlingen-Glass-GBP-Monthly-Calendar-Nov-2026.xlsx
@@ -102,7 +102,8 @@
 Button: Free Estimate</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-02_gbp-post-01_1200x900.png</t>
+    <t xml:space="preserve">2026-11-02_gbp-post-01_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/image00008.jpg</t>
@@ -137,7 +138,8 @@
 Button: Book a Free Inspection</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-03_gbp-post-02_1200x900.png</t>
+    <t xml:space="preserve">2026-11-03_gbp-post-02_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/image00005.jpg</t>
@@ -164,7 +166,8 @@
 Button: Ask Our Team</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-04_gbp-post-03_1200x900.png</t>
+    <t xml:space="preserve">2026-11-04_gbp-post-03_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://unsplash.com/photos/9EyiD1RRYRs (Unsplash licence)</t>
@@ -193,7 +196,8 @@
 Button: Meet the Team</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-05_gbp-post-04_1200x900.png</t>
+    <t xml:space="preserve">2026-11-05_gbp-post-04_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/McAllen-District-Office-12-04-08-001.jpg</t>
@@ -219,7 +223,8 @@
 Button: Free Bathroom Consultation</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-06_gbp-post-05_1200x900.png</t>
+    <t xml:space="preserve">2026-11-06_gbp-post-05_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/IMG_20231208_134141.jpg</t>
@@ -240,7 +245,8 @@
 Button: Compare Styles</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-09_gbp-post-06_1200x900.png</t>
+    <t xml:space="preserve">2026-11-09_gbp-post-06_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/ShowerDoor-scaled.jpg
@@ -265,7 +271,8 @@
 Button: Book a Campus Walkthrough</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-10_gbp-post-07_1200x900.png</t>
+    <t xml:space="preserve">2026-11-10_gbp-post-07_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/Rio-Hondo-Middle-School-3.jpg</t>
@@ -285,7 +292,8 @@
 Button: Free Assessment</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-11_gbp-post-08_1200x900.png</t>
+    <t xml:space="preserve">2026-11-11_gbp-post-08_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/image00003.jpg</t>
@@ -306,7 +314,8 @@
 Button: Free Film Assessment</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-12_gbp-post-09_1200x900.png</t>
+    <t xml:space="preserve">2026-11-12_gbp-post-09_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/Harlingen-Middle-School-Screw-Locations-Ext-Doors-011.jpg</t>
@@ -329,7 +338,8 @@
 Button: Request an Assessment</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-13_gbp-post-10_1200x900.png</t>
+    <t xml:space="preserve">2026-11-13_gbp-post-10_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/IMG_0499-scaled.jpg</t>
@@ -352,7 +362,8 @@
 Button: Ask About Financing</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-16_gbp-post-11_1200x900.png</t>
+    <t xml:space="preserve">2026-11-16_gbp-post-11_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/IMG_20231208_134139.jpg</t>
@@ -375,7 +386,8 @@
 Button: Get a Free Quote</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-17_gbp-post-12_1200x900.png</t>
+    <t xml:space="preserve">2026-11-17_gbp-post-12_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/IMG_20231208_134148.jpg</t>
@@ -395,7 +407,8 @@
 Button: See Coverage</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-18_gbp-post-13_1200x900.png</t>
+    <t xml:space="preserve">2026-11-18_gbp-post-13_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/IMG_20231208_134144.jpg</t>
@@ -415,7 +428,8 @@
 Button: Book a Repair</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-19_gbp-post-14_1200x900.png</t>
+    <t xml:space="preserve">2026-11-19_gbp-post-14_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/IMG_20231208_134134.jpg</t>
@@ -435,7 +449,8 @@
 Button: Free Window Inspection</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-20_gbp-post-15_1200x900.png</t>
+    <t xml:space="preserve">2026-11-20_gbp-post-15_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/IMG_20200123_141554436-scaled.jpg</t>
@@ -455,7 +470,8 @@
 Button: Schedule a Walkthrough</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-23_gbp-post-16_1200x900.png</t>
+    <t xml:space="preserve">2026-11-23_gbp-post-16_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/UTB-Kinesiology-Bldg.jpg</t>
@@ -478,7 +494,8 @@
 Button: Talk to Our Commercial Team</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-24_gbp-post-17_1200x900.png</t>
+    <t xml:space="preserve">2026-11-24_gbp-post-17_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/McAllen-District-Office-12-04-08-002.jpg</t>
@@ -501,7 +518,8 @@
 Button: Book a Visit</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-25_gbp-post-18_1200x900.png</t>
+    <t xml:space="preserve">2026-11-25_gbp-post-18_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://unsplash.com/photos/_enXmoXudAk (Unsplash licence)</t>
@@ -521,7 +539,8 @@
 Button: </t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-26_gbp-post-19_1200x900.png</t>
+    <t xml:space="preserve">2026-11-26_gbp-post-19_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2025/01/fbinfoo-scaled.jpg (cropped)</t>
@@ -541,7 +560,8 @@
 Button: Book Free Consultation</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-27_gbp-post-20_1200x900.png</t>
+    <t xml:space="preserve">2026-11-27_gbp-post-20_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/before.jpg
@@ -565,7 +585,8 @@
 Button: Get a Free Quote</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-11-30_gbp-post-21_1200x900.png</t>
+    <t xml:space="preserve">2026-11-30_gbp-post-21_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/image00009.jpg</t>
@@ -585,7 +606,8 @@
 Button: See Our Projects</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-12-01_gbp-post-22_1200x900.png</t>
+    <t xml:space="preserve">2026-12-01_gbp-post-22_1200x900.png
+(open in Google Drive)</t>
   </si>
   <si>
     <t xml:space="preserve">https://harlingenglass.com/wp-content/uploads/2024/01/45130555_1967058790260758_3379670728264646656_n.jpg
@@ -2836,7 +2858,7 @@
       <c r="L2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="5" t="s">
         <v>22</v>
       </c>
       <c r="N2" s="4" t="s">
@@ -2884,7 +2906,7 @@
       <c r="L3" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="5" t="s">
         <v>32</v>
       </c>
       <c r="N3" s="4" t="s">
@@ -2934,7 +2956,7 @@
       <c r="L4" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="M4" s="4" t="s">
+      <c r="M4" s="5" t="s">
         <v>39</v>
       </c>
       <c r="N4" s="4" t="s">
@@ -2982,7 +3004,7 @@
       <c r="L5" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M5" s="5" t="s">
         <v>47</v>
       </c>
       <c r="N5" s="4" t="s">
@@ -3030,7 +3052,7 @@
       <c r="L6" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="M6" s="5" t="s">
         <v>54</v>
       </c>
       <c r="N6" s="4" t="s">
@@ -3078,7 +3100,7 @@
       <c r="L7" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="M7" s="5" t="s">
         <v>59</v>
       </c>
       <c r="N7" s="4" t="s">
@@ -3126,7 +3148,7 @@
       <c r="L8" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="M8" s="5" t="s">
         <v>65</v>
       </c>
       <c r="N8" s="4" t="s">
@@ -3174,7 +3196,7 @@
       <c r="L9" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="M9" s="5" t="s">
         <v>70</v>
       </c>
       <c r="N9" s="4" t="s">
@@ -3222,7 +3244,7 @@
       <c r="L10" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="M10" s="4" t="s">
+      <c r="M10" s="5" t="s">
         <v>75</v>
       </c>
       <c r="N10" s="4" t="s">
@@ -3270,7 +3292,7 @@
       <c r="L11" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="M11" s="4" t="s">
+      <c r="M11" s="5" t="s">
         <v>81</v>
       </c>
       <c r="N11" s="4" t="s">
@@ -3318,7 +3340,7 @@
       <c r="L12" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="M12" s="5" t="s">
         <v>87</v>
       </c>
       <c r="N12" s="4" t="s">
@@ -3366,7 +3388,7 @@
       <c r="L13" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="M13" s="4" t="s">
+      <c r="M13" s="5" t="s">
         <v>93</v>
       </c>
       <c r="N13" s="4" t="s">
@@ -3414,7 +3436,7 @@
       <c r="L14" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="M14" s="4" t="s">
+      <c r="M14" s="5" t="s">
         <v>98</v>
       </c>
       <c r="N14" s="4" t="s">
@@ -3462,7 +3484,7 @@
       <c r="L15" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="M15" s="4" t="s">
+      <c r="M15" s="5" t="s">
         <v>103</v>
       </c>
       <c r="N15" s="4" t="s">
@@ -3510,7 +3532,7 @@
       <c r="L16" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="M16" s="4" t="s">
+      <c r="M16" s="5" t="s">
         <v>108</v>
       </c>
       <c r="N16" s="4" t="s">
@@ -3558,7 +3580,7 @@
       <c r="L17" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="M17" s="4" t="s">
+      <c r="M17" s="5" t="s">
         <v>113</v>
       </c>
       <c r="N17" s="4" t="s">
@@ -3608,7 +3630,7 @@
       <c r="L18" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="M18" s="4" t="s">
+      <c r="M18" s="5" t="s">
         <v>119</v>
       </c>
       <c r="N18" s="4" t="s">
@@ -3656,7 +3678,7 @@
       <c r="L19" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="M19" s="4" t="s">
+      <c r="M19" s="5" t="s">
         <v>125</v>
       </c>
       <c r="N19" s="4" t="s">
@@ -3704,7 +3726,7 @@
       <c r="L20" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="M20" s="4" t="s">
+      <c r="M20" s="5" t="s">
         <v>130</v>
       </c>
       <c r="N20" s="4" t="s">
@@ -3752,7 +3774,7 @@
       <c r="L21" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="M21" s="4" t="s">
+      <c r="M21" s="5" t="s">
         <v>135</v>
       </c>
       <c r="N21" s="4" t="s">
@@ -3802,7 +3824,7 @@
       <c r="L22" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="M22" s="4" t="s">
+      <c r="M22" s="5" t="s">
         <v>141</v>
       </c>
       <c r="N22" s="4" t="s">
@@ -3850,7 +3872,7 @@
       <c r="L23" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="M23" s="4" t="s">
+      <c r="M23" s="5" t="s">
         <v>146</v>
       </c>
       <c r="N23" s="4" t="s">
@@ -3872,6 +3894,30 @@
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="M2" r:id="rId1" display="2026-11-02_gbp-post-01_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M3" r:id="rId2" display="2026-11-03_gbp-post-02_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M4" r:id="rId3" display="2026-11-04_gbp-post-03_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M5" r:id="rId4" display="2026-11-05_gbp-post-04_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M6" r:id="rId5" display="2026-11-06_gbp-post-05_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M7" r:id="rId6" display="2026-11-09_gbp-post-06_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M8" r:id="rId7" display="2026-11-10_gbp-post-07_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M9" r:id="rId8" display="2026-11-11_gbp-post-08_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M10" r:id="rId9" display="2026-11-12_gbp-post-09_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M11" r:id="rId10" display="2026-11-13_gbp-post-10_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M12" r:id="rId11" display="2026-11-16_gbp-post-11_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M13" r:id="rId12" display="2026-11-17_gbp-post-12_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M14" r:id="rId13" display="2026-11-18_gbp-post-13_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M15" r:id="rId14" display="2026-11-19_gbp-post-14_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M16" r:id="rId15" display="2026-11-20_gbp-post-15_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M17" r:id="rId16" display="2026-11-23_gbp-post-16_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M18" r:id="rId17" display="2026-11-24_gbp-post-17_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M19" r:id="rId18" display="2026-11-25_gbp-post-18_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M20" r:id="rId19" display="2026-11-26_gbp-post-19_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M21" r:id="rId20" display="2026-11-27_gbp-post-20_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M22" r:id="rId21" display="2026-11-30_gbp-post-21_1200x900.png&#10;(open in Google Drive)"/>
+    <hyperlink ref="M23" r:id="rId22" display="2026-12-01_gbp-post-22_1200x900.png&#10;(open in Google Drive)"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3879,7 +3925,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId23"/>
 </worksheet>
 </file>
 

</xml_diff>